<commit_message>
Add apertura 142/143/144 coded passages to QDA corpus (rows 78-98)
</commit_message>
<xml_diff>
--- a/analysis/results/qda_v3_coded_corpus_v3.xlsx
+++ b/analysis/results/qda_v3_coded_corpus_v3.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coded Passages" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Freq — By Dimension" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Freq — By Sub-code" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Speech Overview" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Coded Passages" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Freq — By Dimension" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Freq — By Sub-code" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Speech Overview" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Coded Passages'!$A$2:$J$70</definedName>
@@ -462,14 +462,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -491,8 +491,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -511,10 +511,10 @@
             <v>D1.1</v>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="3B82F6"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="3B82F6"/>
               </a:solidFill>
@@ -525,16 +525,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -616,10 +616,10 @@
             <v>D1.2</v>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="F59E0B"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="F59E0B"/>
               </a:solidFill>
@@ -630,16 +630,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -721,10 +721,10 @@
             <v>D1.3</v>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="EF4444"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="EF4444"/>
               </a:solidFill>
@@ -735,16 +735,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -826,10 +826,10 @@
             <v>D2.2</v>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="06B6D4"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="06B6D4"/>
               </a:solidFill>
@@ -840,16 +840,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -931,10 +931,10 @@
             <v>D2.3</v>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="8B5CF6"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="8B5CF6"/>
               </a:solidFill>
@@ -945,16 +945,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -1036,10 +1036,10 @@
             <v>IND</v>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="9CA3AF"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="9CA3AF"/>
               </a:solidFill>
@@ -1050,16 +1050,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -1157,9 +1157,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -1181,8 +1181,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1193,7 +1193,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1202,9 +1202,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1236,7 +1236,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -1248,9 +1248,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -1272,8 +1272,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1284,7 +1284,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1293,9 +1293,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1320,16 +1320,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1350,10 +1350,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1365,14 +1365,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1394,8 +1394,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1422,10 +1422,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1433,16 +1433,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -1541,7 +1541,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1550,9 +1550,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1584,7 +1584,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -1598,7 +1598,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1607,9 +1607,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1634,16 +1634,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1664,10 +1664,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1679,14 +1679,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1708,8 +1708,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1736,10 +1736,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1747,16 +1747,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -1937,9 +1937,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -1961,8 +1961,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1973,7 +1973,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1982,9 +1982,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2016,7 +2016,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2028,9 +2028,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2052,8 +2052,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2064,7 +2064,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2073,9 +2073,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2100,16 +2100,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2130,10 +2130,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2145,14 +2145,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2174,8 +2174,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="3B82F6"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2312,10 +2312,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="8B5CF6"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2323,16 +2323,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2429,9 +2429,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2453,8 +2453,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2465,7 +2465,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2474,9 +2474,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2508,7 +2508,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2520,9 +2520,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2544,8 +2544,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2556,7 +2556,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2565,9 +2565,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2592,16 +2592,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2622,10 +2622,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2637,7 +2637,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -2657,9 +2657,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2684,9 +2684,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2696,7 +2696,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -2716,9 +2716,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2728,7 +2728,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -2748,9 +2748,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2942,7 +2942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J100"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.25"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -6863,6 +6863,1056 @@
       <c r="J79" s="45" t="inlineStr">
         <is>
           <t>Davos · Speech</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>78</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>D1.2</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Attack on Universities</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>D1.2 — Public Science &amp; Expertise</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Attack on Universities</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>En el plano de la Educación Superior, la creación de universidades se ha convertido en un negocio más de la política y en los profesorados e institutos de formación inicial de docentes se imparte, cada vez más, adoctrinamiento político, en lugar de educación.</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Milei frames teacher-training colleges and universities as sites of "political indoctrination" rather than education, attacking the epistemic infrastructure that produces Argentina's scientific and professional classes. This delegitimizes the knowledge-producing institutions most responsible for environmental and sustainability expertise, positioning academic education as a captured ideological project rather than a reliable source of expertise for policymaking. The move is structural rather than specific: it does not name individual environmental scholars but pathologizes the institutional culture from which climate-relevant expertise emerges.</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Apertura 142 (2024)</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>2024-03-01</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>79</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>D1.1</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Anti-Casta (Elite Frame)</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>D1.1 — State Intervention &amp; Governance</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Anti-Casta (Elite Frame)</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Tras haber visto con mis propios ojos y en detalle la vulgaridad del despilfarro con el que la política se acostumbró a vivir, ratifico una vez más que la casta política es lo peor que le puede pasar a un país como el nuestro.</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Milei confirms and intensifies the "la casta" frame as the foundational political category of his governing project. This is the first explicit formalization of the casta indictment in a presidential address, establishing the frame that will subsequently be applied to environmental agencies, sustainability technocrats, and international governance bodies. When this same anti-casta rhetoric is deployed later against CONICET, the Ministry of Environment, or multilateral climate bodies, its legitimating logic has been institutionalized here in the opening address of his presidency.</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Apertura 142 (2024)</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>2024-03-01</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>80</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>D1.1</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Deregulation Benefits</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>D1.1 — State Intervention &amp; Governance</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Deregulation Benefits</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Por último, también firmamos un mega Decreto de Necesidad y Urgencia para, por primera vez en décadas, devolverles la libertad a los argentinos en vez de quitárselas con regulaciones sin sentido.</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>The DNU 70/23 -- framed here as "returning freedom" to Argentines -- included the derogation of dozens of environmental and land-use regulations, alongside broader economic deregulation. By presenting the entire deregulatory package as "freedom from senseless regulations," Milei establishes the foundational rhetorical move that makes environmental regulation categorically illegitimate: not harmful to growth per se, but a deprivation of liberty. The positive framing ("returning freedom") is analytically central -- it does not argue against regulations on techno-economic grounds but on moral-liberty grounds.</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Apertura 142 (2024)</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>2024-03-01</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>81</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>D1.1</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Delegitimization of Regulation</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>D1.1 — State Intervention &amp; Governance</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Delegitimization of Regulation</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Por último, también firmamos un mega Decreto de Necesidad y Urgencia para, por primera vez en décadas, devolverles la libertad a los argentinos en vez de quitárselas con regulaciones sin sentido.</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>The phrase "regulaciones sin sentido" does categorical ideological work: it asserts that regulations as a class are senseless, without needing to evaluate any specific regulation's rationale. This is not a technocratic critique but an a priori dismissal -- the state's power to regulate is itself illegitimate. Environmental and sustainability regulations, which depend on public justification of market failures and externalities, are pre-emptively categorized as "senseless" by this framing, before any specific environmental case can be made.</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Apertura 142 (2024)</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>2024-03-01</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>82</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>D1.1</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Anti-State / Anti-Bureaucratic</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>D1.1 — State Intervention &amp; Governance</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Anti-State / Anti-Bureaucratic</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Eliminamos cajas de militancia como el INCAA, el INADI, el Ministerio de la Mujer y Télam y volvimos superavitarias empresas emblemáticas de la militancia deficitaria, como Aerolíneas Argentinas, AySA, Intercargo y ENARSA.</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>The explicit grouping of INCAA, INADI, and the Ministerio de la Mujer as "cajas de militancia" establishes the rhetorical pattern of labeling progressive-adjacent state institutions as corrupt political patronage rather than legitimate public functions. INADI and the women's ministry represent precisely the kind of social-regulatory institutions that also administer environmental and sustainability policy -- agencies whose authority rests on normative social science rather than market metrics. Categorizing them as inherently militant/patronage-driven pre-emptively applies the same frame to environmental agencies.</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Apertura 143 (2025)</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>2025-03-01</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>83</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>D1.1</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Market Primacy</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>D1.1 — State Intervention &amp; Governance</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Market Primacy</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Además, eliminamos la obra pública --que era uno de los curros más grandes de la política--. [...] la obra pública no genera trabajo, la obra pública genera impuestos.</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>The sustained argument that public works are a net economic negative because they crowd out private spending is a classic market-primacy move with direct implications for climate governance. Climate transition policy relies substantially on public investment -- green infrastructure, renewable energy buildout, adaptation works. By asserting categorically that public investment destroys value rather than creating it, this passage delegitimizes the economic logic of public climate investment before any specific environmental case can be made. The framing also pathologizes public expenditure on infrastructure as inherently corrupt ("curro de la política"), making it politically toxic for future governments to justify green public investment.</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Apertura 143 (2025)</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>2025-03-01</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>84</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>D1.1</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Deregulation Benefits</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>D1.1 — State Intervention &amp; Governance</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Deregulation Benefits</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>hemos concentrado alrededor y concretado 1700 reformas estructurales, eliminando regulaciones que cercenaban libertades comerciales y económicas y le ponían palos en la rueda al gran motor productivo de nuestro país, que es el sector privado.</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>The "1700 structural reforms" figure is presented as the central achievement of the first year, with deregulation framed as "removing sticks from the wheels" of the productive sector. The institutionalization of a dedicated "Ministro de Desregulación" makes deregulation a permanent administrative function of the state, not a one-time corrective. This is significant for climate governance because environmental regulations constitute a substantial portion of the regulatory corpus being dismantled; the weight-of-paper metaphor trivializes regulatory content by reducing regulations to their bureaucratic bulk rather than their protective function.</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Apertura 143 (2025)</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>2025-03-01</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>85</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>D1.1</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Deregulation Benefits</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>D1.1 — State Intervention &amp; Governance</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Deregulation Benefits</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>No es menor lo de Elon con la motosierra. La motosierra, hoy, es un símbolo de cambio de época y el inicio de una nueva era dorada para la humanidad, pero esta vez, en vez de ir a contramano del mundo, Argentina está a la vanguardia del mundo.</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>The explicit alignment of Milei's chainsaw symbol with Elon Musk's DOGE deregulatory operation is a transnational validation move: it frames the anti-regulatory revolution as a global historical trend ("a new golden era for humanity") in which Argentina is the vanguard. This is significant for climate governance because both DOGE and Milei's deregulatory agenda specifically targeted environmental agencies and regulations. The "new golden era" framing positions environmental deregulation not as a contested political choice but as the natural direction of history -- a form of temporal determinism that makes resistance to deregulation appear backward.</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Apertura 143 (2025)</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>2025-03-01</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>86</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>D1.1</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Rejection of Multilateral Governance</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>D1.1 — State Intervention &amp; Governance</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Rejection of Multilateral Governance</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>es necesario estar dispuesto a flexibilizar o, incluso, llegado el caso, a salir del Mercosur, que lo único que logró desde su creación es enriquecer a los grandes industriales brasileros a costa de empobrecer a los argentinos.</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>The willingness to exit Mercosur -- a major regional multilateral governance framework -- is framed as a necessary condition for national prosperity. Mercosur's institutional architecture includes environmental and sustainability chapters, and its relationship with the EU (being negotiated at this time) involved environmental conditionality. By treating Mercosur exit as a legitimate policy option and framing multilateral economic integration as inherently enriching other countries at Argentina's expense, Milei extends the rejection-of-multilateral-governance logic from the climate domain (2030 Agenda, IPCC) to the broader institutional architecture of regional governance.</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Apertura 143 (2025)</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>2025-03-01</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>87</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>D1.3</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Woke Bundling</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>D1.3 — Cultural Backlash</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Woke Bundling</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>tenemos que recuperar el imperio de la igualdad ante la ley, terminando con este sistema de cupos de distinto tipo que impone desde a quién emplear hasta a quién votar. Hemos llegado al punto en el que hay cupos hasta para emplear gente en medios de comunicación o para la programación de artistas en un festival.</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>The grouping of employment quotas (gender, diversity), media programming quotas, and electoral quotas under a single "equality-before-the-law" critique performs ideological bundling: it treats affirmative representation mechanisms as a unified progressive excess. The phrase "ciertos grupos percibidos como oprimidos" explicitly frames identity-based policy as based on perception rather than material reality -- the same epistemic move used to frame climate science as perception-based rather than empirically grounded. The anti-quota framing extends the anti-"woke" frame into public institutions, preparing the terrain for applying the same logic to environmental quotas, emissions targets, and international reporting obligations.</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Apertura 143 (2025)</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>2025-03-01</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>88</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>D1.3</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Civilizational Defense</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>D1.3 — Cultural Backlash</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Civilizational Defense</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>en nuestra visión existe un claro orden de mérito. En primer lugar, están la ética y la moral en base a los valores de Occidente. Esto es, la filosofía griega, el derecho romano, la rectitud de los estoicos y los valores judeocristianos. En segundo lugar, ubicamos la eficiencia económica. Y, por último, en tercer lugar, el utilitarismo político.</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>The explicit ordering of moral values -- Western ethics/morality first, economic efficiency second, political utilitarianism third -- establishes a normative hierarchy in which "Occidente" (Greek philosophy, Roman law, Judeo-Christian values) is the foundational reference for all legitimate policy. Sustainability governance and environmental science, which invoke collective/intergenerational obligations that cut across individual rights, are implicitly subordinate to this Western-individual-rights framework. Climate policy that invokes the 2030 Agenda or IPCC consensus falls outside the "moral" primary category by definition -- it would be classified as "utilitarismo político" at best.</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Apertura 144 (2026)</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>89</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>D1.1</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Deregulation Benefits</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>D1.1 — State Intervention &amp; Governance</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Deregulation Benefits</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>El primer pilar es la desregulación de la economía. Esta política de exterminar regulaciones no solo es una forma de restaurar el derecho de propiedad, sino que además libera rendimientos crecientes, los cuales son la base del crecimiento económico. Si no asimilamos este punto, todo lo demás será en vano.</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>The framing of deregulation as "exterminar regulaciones" -- exterminating rather than reforming regulations -- uses maximalist language that positions the regulatory corpus itself as a hostile entity to be eliminated rather than a governance tool to be calibrated. The positive theoretical claim -- deregulation "liberates increasing returns," which is the basis for economic growth -- forecloses the case for environmental regulation before it can be made: if regulations by definition suppress increasing returns and therefore growth, then environmental regulations are anti-growth by definition, and any empirical case for environmental regulation would be dismissed as theoretically unfounded.</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Apertura 144 (2026)</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>90</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>D1.1</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Sustainability as Ideological or Harmful</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>D1.1 — State Intervention &amp; Governance</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Sustainability as Ideological or Harmful</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Vamos a construir un marco legal robusto que permita el desarrollo primario para beneficio de todos los argentinos, con cuidados, pero lejos de prejuicios ambientalistas absurdos. Me refiero a todos los recursos: a los minerales críticos como el cobre y el litio, a la pesca y a la agricultura, a los hidrocarburos convencionales y no convencionales, a las economías regionales y al sector agropecuario.</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>The phrase "lejos de prejuicios ambientalistas absurdos" is the most explicit climate-governance delegitimation passage in the apertura corpus. By framing environmental concerns as "absurd prejudices" in the specific context of announcing legislative removal of legal barriers to resource extraction (hydrocarbon, mining, agro), Milei acknowledges the existence of environmental concerns while categorically dismissing their epistemic status. "Prejuicios" frames environmentalism as pre-rational bias rather than evidence-based concern, and "absurdos" intensifies this by asserting their irrationality is self-evident. This is a stronger dismissal than most previous coded passages, which tended to delegitimize environmental governance indirectly.</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Apertura 144 (2026)</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>91</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>D1.1</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Delegitimization of Regulation</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>D1.1 — State Intervention &amp; Governance</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Delegitimization of Regulation</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>vamos a buscar remover las barreras legales que se interponen entre la sociedad y su riqueza. Vamos a construir un marco legal robusto que permita el desarrollo primario para beneficio de todos los argentinos, con cuidados, pero lejos de prejuicios ambientalistas absurdos.</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>The explicit goal of "remover las barreras legales que se interponen entre la sociedad y su riqueza" -- applied to hydrocarbon extraction, mining, fishing, and agriculture -- frames environmental and resource-protection regulations as barriers between society and its wealth rather than as legitimate governance of common resources. This is a property-rights argument against environmental regulation: natural resources are society's "wealth," regulations are "barriers," and removing them is restoration of rightful access. The enumeration of all primary sectors (conventional and non-conventional hydrocarbons, critical minerals, fishing, agro) establishes the comprehensive scope of the deregulatory intention.</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Apertura 144 (2026)</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>92</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>D1.3</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Civilizational Defense</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>D1.3 — Cultural Backlash</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Civilizational Defense</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Dedicaremos este año a examinar la organización jurídica e institucional que nos trajo hasta aquí y construir una arquitectura nueva; la arquitectura que tendrá el Estado argentino los próximos 50 años, teniendo la moral occidental como política de estado.</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>The declaration that "la moral occidental" will be the guiding policy framework for the next 50 years of Argentine statehood is the most expansive civilizational claim in the corpus. By anchoring the 50-year institutional architecture in "Western morality" rather than in constitutional norms or democratic consensus, Milei positions any future climate governance framework that invokes collective obligations, international agreements, or IPCC expert consensus as fundamentally incompatible with this foundational moral architecture. The 50-year horizon attempts to make the libertarian-Western framework normatively permanent, pre-empting future democratic mandates for climate governance.</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Apertura 144 (2026)</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>93</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>D1.1</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Rejection of Multilateral Governance</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>D1.1 — State Intervention &amp; Governance</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Rejection of Multilateral Governance</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>La era de la cooperación global sin brújula moral ha terminado. Entramos a una nueva era de grandes naciones que compiten por asegurarse cadenas de valor verticales.</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>The declaration that "the era of global cooperation without moral compass has ended" is the most direct rejection of multilateral governance in the apertura corpus. Global cooperation without moral compass refers precisely to the multilateral governance architecture -- the UN system, the IPCC, the 2030 Agenda, the Paris Agreement -- which Milei's framework identifies as lacking the "moral compass" of Western individual-rights values. The "new era" of competing great nations replacing cooperative global governance is structurally incompatible with the climate governance regime, which depends on multilateral cooperation and compliance commitments.</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Apertura 144 (2026)</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>94</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>D1.1</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Market Primacy</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>D1.1 — State Intervention &amp; Governance</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Market Primacy</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Tenemos los minerales críticos que necesita Occidente, tenemos la energía: gas, petróleo, energía nuclear y energía renovable para abastecer cadenas de producción de escala.</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>The framing of Argentina's natural resources -- including gas, petróleo (conventional and unconventional), and nuclear energy alongside renewables -- as strategic assets serving "Occidente" positions fossil fuel extraction as geopolitically necessary and morally justified. By listing fossil fuels and renewables together without distinction under Argentina's strategic resource profile, this passage neutralizes the climate-energy transition narrative: all energy resources are equally valuable as Occidental strategic assets, and the distinction between high-carbon and low-carbon energy (central to climate policy) is irrelevant in the market/geopolitical frame.</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Apertura 144 (2026)</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>95</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>D1.1</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Anti-Casta (Elite Frame)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>D1.1 — State Intervention &amp; Governance</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Anti-Casta (Elite Frame)</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>el mundo solo tiene dos tipos de personas. Los que viven de lo que otros producen, es decir, los parásitos --o sea, ustedes--, y los que producen todo lo que hace posible la vida moderna. Mientras ustedes redactan regulaciones, nosotros creamos riqueza; mientras ustedes prometen igualdad, nosotros generamos prosperidad; mientras ustedes reparten pobreza, nosotros multiplicamos la abundancia.</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>The Huerta de Soto quote -- introduced by the President and applied directly to the congressional opposition -- delivers the parasites/producers binary in its most philosophically elaborated form. Environmental regulators, sustainability agencies, and scientific advisory bodies all "draft regulations" in Huerta de Soto's formulation, making them unambiguously parasites rather than producers in this moral framework. The anti-casta frame is here given its strongest moral-ontological expression: not simply that politicians are corrupt, but that the regulatory state -- those who "draft regulations" -- is structurally parasitic on the productive sector.</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Apertura 144 (2026)</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>96</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>D1.3</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Neo-Marxism</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>D1.3 — Cultural Backlash</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Neo-Marxism</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>La verdadera batalla de nuestro tiempo es cultural, filosófica y moral. Es elegir el sistema que sacó de la pobreza a millones. Es para dejar de ser una Nación inmadura, que dilapida el futuro para repartir beneficios en el presente; y convertirnos en una nación madura, que planifica las reglas de juego para que haya presente y futuro.</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>The framing of "la verdadera batalla de nuestro tiempo" as cultural, philosophical, and moral -- a battle between capitalism and socialism/collectivism -- is the Neo_Marxism code at its most developed. The climate governance regime is implicitly on the collectivist side: it involves state planning, expert mediation, and redistribution of present consumption toward future generations. The "nación madura que planifica para presente y futuro" simultaneously appropriates sustainability's intergenerational language and redeploys it against climate policy.</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Apertura 144 (2026)</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>97</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>IND</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Temporal Appropriation</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Inductive</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Temporal Appropriation</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Es para dejar de ser una Nación inmadura, que dilapida el futuro para repartir beneficios en el presente; y convertirnos en una nación madura, que planifica las reglas de juego para que haya presente y futuro; y para que cada ciudadano pueda elegir libremente su propio destino.</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>The contrast between a "nación inmadura que dilapida el futuro para repartir beneficios en el presente" and a "nación madura que planifica las reglas de juego para que haya presente y futuro" inverts the sustainability discourse's intergenerational frame. Climate governance's core moral claim is that present consumption sacrifices the future; here Milei appropriates that moral structure to argue that state redistribution (including sustainability programs) is what sacrifices the future, while market freedom is what "plans for both present and future." This is the fourth confirmed corpus instance of Temporal_Appropriation, exceeding the formalization threshold of 2+ appearances.</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Apertura 144 (2026)</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>98</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>D1.1</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Anti-State / Anti-Bureaucratic</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>D1.1 — State Intervention &amp; Governance</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Anti-State / Anti-Bureaucratic</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>El Estado presente, que pretende hacerse cargo de todos los órdenes de la vida, fracasó. Por eso necesitamos un Estado ágil, abocado a unas pocas funciones esenciales, sintetizadas en la defensa de la vida, la libertad y la propiedad privada, amparado en lo que definimos, como decía Ayn Rand, la ética de la emergencia.</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>The invocation of Ayn Rand's "ethics of emergency" to justify a minimal state, combined with the claim that any state "that pretends to take care of all dimensions of life" has failed, is a direct repudiation of the regulatory state's legitimacy in the domain of climate governance. Climate governance requires precisely the kind of state that "pretends to take care" of long-range collective problems that markets do not spontaneously resolve. By framing state scope as the cause of failure (rather than specific bad policies), Milei pre-emptively delegitimizes any future government's attempt to use state capacity for environmental management.</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Apertura 144 (2026)</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Buenos Aires · Apertura</t>
         </is>
       </c>
     </row>

</xml_diff>